<commit_message>
Library Update. Project settings update.
</commit_message>
<xml_diff>
--- a/docs/WorkingStatus.xlsx
+++ b/docs/WorkingStatus.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kitoh\source\repos\aliceconv\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303D676E-6DB0-4093-9C0B-D7FDF1DE3475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F10BF06-539F-40FF-86E9-82744A247273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" activeTab="2" xr2:uid="{FF061521-1F21-4413-9E31-090A18910087}"/>
+    <workbookView xWindow="2010" yWindow="690" windowWidth="26535" windowHeight="16770" activeTab="2" xr2:uid="{FF061521-1F21-4413-9E31-090A18910087}"/>
   </bookViews>
   <sheets>
     <sheet name="CG" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="115">
   <si>
     <t>リトルプリンセス</t>
   </si>
@@ -421,6 +421,62 @@
   </si>
   <si>
     <t>Scenario</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-0</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-0m</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-1g</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>×</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-0</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>`</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-2d</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-3</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-2r</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-2rx</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-3t</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-3(なぐりまくりたわぁ -3t)</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -453,7 +509,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -463,6 +519,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -481,7 +555,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -496,6 +570,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1373,7 +1471,7 @@
       <c r="G38" t="s">
         <v>56</v>
       </c>
-      <c r="H38" t="s">
+      <c r="H38" s="3" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1390,6 +1488,7 @@
       <c r="G39" t="s">
         <v>55</v>
       </c>
+      <c r="H39" s="3"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
@@ -1599,7 +1698,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="H38:H39"/>
     <mergeCell ref="G33:G34"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="E12:F12"/>
@@ -1720,25 +1820,49 @@
       <c r="A9" t="s">
         <v>0</v>
       </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>1</v>
       </c>
+      <c r="B10" s="8" t="s">
+        <v>106</v>
+      </c>
       <c r="C10" t="s">
         <v>98</v>
       </c>
       <c r="D10" t="s">
         <v>99</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>2</v>
       </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
       <c r="D11" t="s">
         <v>99</v>
       </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
@@ -1762,11 +1886,15 @@
       <c r="G12" t="s">
         <v>94</v>
       </c>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>4</v>
       </c>
+      <c r="B13" s="8"/>
+      <c r="H13" s="7"/>
       <c r="I13" t="s">
         <v>94</v>
       </c>
@@ -1775,15 +1903,20 @@
       <c r="A14" t="s">
         <v>5</v>
       </c>
+      <c r="B14" s="7"/>
       <c r="C14" t="s">
         <v>98</v>
       </c>
       <c r="D14" t="s">
         <v>97</v>
       </c>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
       <c r="G14" t="s">
         <v>94</v>
       </c>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
@@ -1792,6 +1925,7 @@
       <c r="B15" t="s">
         <v>96</v>
       </c>
+      <c r="C15" s="7"/>
       <c r="D15" t="s">
         <v>97</v>
       </c>
@@ -1804,6 +1938,8 @@
       <c r="G15" t="s">
         <v>94</v>
       </c>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
@@ -1827,6 +1963,8 @@
       <c r="G16" t="s">
         <v>94</v>
       </c>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
@@ -1850,6 +1988,8 @@
       <c r="G17" t="s">
         <v>94</v>
       </c>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
@@ -1858,12 +1998,17 @@
       <c r="B18" t="s">
         <v>96</v>
       </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
       <c r="E18" t="s">
         <v>96</v>
       </c>
       <c r="F18" t="s">
         <v>94</v>
       </c>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
@@ -1887,6 +2032,8 @@
       <c r="G19" t="s">
         <v>94</v>
       </c>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
@@ -1896,6 +2043,7 @@
         <v>94</v>
       </c>
       <c r="C20" s="3"/>
+      <c r="D20" s="7"/>
       <c r="E20" t="s">
         <v>96</v>
       </c>
@@ -1905,6 +2053,8 @@
       <c r="G20" t="s">
         <v>67</v>
       </c>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
@@ -1913,6 +2063,7 @@
       <c r="B21" t="s">
         <v>94</v>
       </c>
+      <c r="C21" s="7"/>
       <c r="D21" t="s">
         <v>97</v>
       </c>
@@ -1925,6 +2076,8 @@
       <c r="G21" t="s">
         <v>94</v>
       </c>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
@@ -1933,12 +2086,16 @@
       <c r="B22" t="s">
         <v>94</v>
       </c>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
       <c r="E22" t="s">
         <v>96</v>
       </c>
+      <c r="F22" s="7"/>
       <c r="G22" t="s">
         <v>94</v>
       </c>
+      <c r="H22" s="7"/>
       <c r="I22" t="s">
         <v>95</v>
       </c>
@@ -1950,12 +2107,17 @@
       <c r="B23" t="s">
         <v>94</v>
       </c>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
       <c r="E23" t="s">
         <v>96</v>
       </c>
+      <c r="F23" s="7"/>
       <c r="G23" t="s">
         <v>94</v>
       </c>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
@@ -1964,6 +2126,7 @@
       <c r="B24" t="s">
         <v>94</v>
       </c>
+      <c r="C24" s="7"/>
       <c r="D24" t="s">
         <v>97</v>
       </c>
@@ -1976,17 +2139,25 @@
       <c r="G24" t="s">
         <v>94</v>
       </c>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>14</v>
       </c>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
       <c r="E25" t="s">
         <v>96</v>
       </c>
+      <c r="F25" s="7"/>
       <c r="G25" t="s">
         <v>94</v>
       </c>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
@@ -1995,12 +2166,17 @@
       <c r="B26" t="s">
         <v>86</v>
       </c>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
       <c r="E26" t="s">
         <v>86</v>
       </c>
+      <c r="F26" s="7"/>
       <c r="G26" t="s">
         <v>86</v>
       </c>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
@@ -2009,12 +2185,17 @@
       <c r="B27" t="s">
         <v>86</v>
       </c>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
       <c r="E27" t="s">
         <v>86</v>
       </c>
+      <c r="F27" s="7"/>
       <c r="G27" t="s">
         <v>86</v>
       </c>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
@@ -2023,6 +2204,7 @@
       <c r="B28" t="s">
         <v>94</v>
       </c>
+      <c r="C28" s="7"/>
       <c r="D28" t="s">
         <v>97</v>
       </c>
@@ -2035,6 +2217,8 @@
       <c r="G28" t="s">
         <v>94</v>
       </c>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
@@ -2043,12 +2227,17 @@
       <c r="B29" t="s">
         <v>86</v>
       </c>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
       <c r="E29" t="s">
         <v>86</v>
       </c>
+      <c r="F29" s="7"/>
       <c r="G29" t="s">
         <v>86</v>
       </c>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
@@ -2057,9 +2246,15 @@
       <c r="B30" t="s">
         <v>86</v>
       </c>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
       <c r="E30" t="s">
         <v>86</v>
       </c>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
@@ -2068,20 +2263,32 @@
       <c r="B31" t="s">
         <v>86</v>
       </c>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
       <c r="E31" t="s">
         <v>86</v>
       </c>
+      <c r="F31" s="7"/>
       <c r="G31" t="s">
         <v>86</v>
       </c>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>21</v>
       </c>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
       <c r="G32" t="s">
         <v>86</v>
       </c>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
@@ -2090,12 +2297,17 @@
       <c r="B33" t="s">
         <v>86</v>
       </c>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
       <c r="E33" t="s">
         <v>86</v>
       </c>
+      <c r="F33" s="7"/>
       <c r="G33" s="3" t="s">
         <v>86</v>
       </c>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
@@ -2104,10 +2316,15 @@
       <c r="B34" t="s">
         <v>86</v>
       </c>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
       <c r="E34" t="s">
         <v>86</v>
       </c>
+      <c r="F34" s="7"/>
       <c r="G34" s="3"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
@@ -2116,9 +2333,15 @@
       <c r="B35" t="s">
         <v>87</v>
       </c>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
       <c r="G35" t="s">
         <v>87</v>
       </c>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
@@ -2127,20 +2350,31 @@
       <c r="B36" t="s">
         <v>86</v>
       </c>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
       <c r="E36" t="s">
         <v>86</v>
       </c>
+      <c r="F36" s="7"/>
       <c r="G36" t="s">
         <v>86</v>
       </c>
       <c r="H36" t="s">
         <v>89</v>
       </c>
+      <c r="I36" s="7"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>26</v>
       </c>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
@@ -2149,15 +2383,19 @@
       <c r="B38" t="s">
         <v>86</v>
       </c>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
       <c r="E38" t="s">
         <v>86</v>
       </c>
+      <c r="F38" s="7"/>
       <c r="G38" t="s">
         <v>86</v>
       </c>
-      <c r="H38" t="s">
+      <c r="H38" s="3" t="s">
         <v>90</v>
       </c>
+      <c r="I38" s="7"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
@@ -2166,12 +2404,17 @@
       <c r="B39" t="s">
         <v>86</v>
       </c>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
       <c r="E39" t="s">
         <v>67</v>
       </c>
+      <c r="F39" s="7"/>
       <c r="G39" t="s">
         <v>86</v>
       </c>
+      <c r="H39" s="3"/>
+      <c r="I39" s="7"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
@@ -2180,9 +2423,15 @@
       <c r="B40" t="s">
         <v>86</v>
       </c>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
       <c r="G40" t="s">
         <v>86</v>
       </c>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
@@ -2191,9 +2440,15 @@
       <c r="B41" t="s">
         <v>86</v>
       </c>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
       <c r="G41" t="s">
         <v>86</v>
       </c>
+      <c r="H41" s="7"/>
+      <c r="I41" s="7"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
@@ -2202,15 +2457,19 @@
       <c r="B42" t="s">
         <v>86</v>
       </c>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
       <c r="E42" t="s">
         <v>86</v>
       </c>
+      <c r="F42" s="7"/>
       <c r="G42" t="s">
         <v>86</v>
       </c>
       <c r="H42" t="s">
         <v>91</v>
       </c>
+      <c r="I42" s="7"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
@@ -2219,9 +2478,12 @@
       <c r="B43" t="s">
         <v>86</v>
       </c>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
       <c r="E43" t="s">
         <v>86</v>
       </c>
+      <c r="F43" s="7"/>
       <c r="G43" t="s">
         <v>86</v>
       </c>
@@ -2236,9 +2498,15 @@
       <c r="B44" t="s">
         <v>86</v>
       </c>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
       <c r="H44" t="s">
         <v>92</v>
       </c>
+      <c r="I44" s="7"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
@@ -2247,9 +2515,15 @@
       <c r="B45" t="s">
         <v>86</v>
       </c>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
       <c r="G45" t="s">
         <v>67</v>
       </c>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
@@ -2258,6 +2532,11 @@
       <c r="B46" t="s">
         <v>86</v>
       </c>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
       <c r="H46" t="s">
         <v>89</v>
       </c>
@@ -2269,6 +2548,11 @@
       <c r="B47" t="s">
         <v>86</v>
       </c>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
       <c r="H47" t="s">
         <v>93</v>
       </c>
@@ -2277,6 +2561,12 @@
       <c r="A48" t="s">
         <v>38</v>
       </c>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
       <c r="J48" t="s">
         <v>86</v>
       </c>
@@ -2288,6 +2578,11 @@
       <c r="B49" t="s">
         <v>86</v>
       </c>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
       <c r="H49" t="s">
         <v>74</v>
       </c>
@@ -2299,6 +2594,11 @@
       <c r="B50" t="s">
         <v>86</v>
       </c>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
       <c r="H50" t="s">
         <v>74</v>
       </c>
@@ -2310,6 +2610,11 @@
       <c r="B51" t="s">
         <v>86</v>
       </c>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
       <c r="H51" t="s">
         <v>74</v>
       </c>
@@ -2321,6 +2626,11 @@
       <c r="B52" t="s">
         <v>86</v>
       </c>
+      <c r="C52" s="7"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7"/>
       <c r="H52" t="s">
         <v>74</v>
       </c>
@@ -2329,6 +2639,12 @@
       <c r="A53" t="s">
         <v>42</v>
       </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
       <c r="H53" t="s">
         <v>88</v>
       </c>
@@ -2340,6 +2656,10 @@
       <c r="B54" t="s">
         <v>86</v>
       </c>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
       <c r="G54" t="s">
         <v>86</v>
       </c>
@@ -2351,6 +2671,12 @@
       <c r="A55" t="s">
         <v>45</v>
       </c>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
@@ -2359,6 +2685,11 @@
       <c r="B56" t="s">
         <v>86</v>
       </c>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
       <c r="H56" t="s">
         <v>77</v>
       </c>
@@ -2367,6 +2698,12 @@
       <c r="A57" t="s">
         <v>44</v>
       </c>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
       <c r="J57" t="s">
         <v>87</v>
       </c>
@@ -2378,9 +2715,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="G33:G34"/>
+    <mergeCell ref="H38:H39"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2390,7 +2728,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42696DDD-9955-4569-87FB-5C3937DD1FF3}">
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="48.875" customWidth="1"/>
@@ -2493,261 +2831,1113 @@
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="D9" t="s">
+      <c r="B9" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="5" t="s">
         <v>57</v>
       </c>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>1</v>
       </c>
-      <c r="D10" t="s">
-        <v>56</v>
-      </c>
+      <c r="B10" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>2</v>
       </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>3</v>
       </c>
+      <c r="B12" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H12" s="9"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>4</v>
       </c>
+      <c r="B13" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="9"/>
+      <c r="I13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>5</v>
       </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>6</v>
       </c>
+      <c r="B15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H15" s="9"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B16" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H16" s="9"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B17" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" s="9"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B18" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="3"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B19" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" s="9"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="3"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B20" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H20" s="9"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B21" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="9"/>
+      <c r="D21" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H21" s="9"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B22" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F22" s="9"/>
+      <c r="G22" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H22" s="9"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B23" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F23" s="9"/>
+      <c r="G23" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H23" s="9"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B24" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" s="9"/>
+      <c r="D24" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H24" s="9"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H25" s="9"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B26" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F26" s="9"/>
+      <c r="G26" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H26" s="9"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="5"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B27" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F27" s="9"/>
+      <c r="G27" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H27" s="9"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B28" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" s="9"/>
+      <c r="D28" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H28" s="9"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B29" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F29" s="9"/>
+      <c r="G29" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H29" s="9"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B30" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B31" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F31" s="9"/>
+      <c r="G31" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H31" s="9"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="5"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H32" s="9"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>22</v>
       </c>
-      <c r="G33" s="3"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B33" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F33" s="9"/>
+      <c r="G33" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H33" s="9"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
-      <c r="G34" s="3"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B34" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F34" s="9"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="L34" s="5"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B35" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H35" s="9"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+      <c r="L35" s="5"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B36" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F36" s="9"/>
+      <c r="G36" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+      <c r="L36" s="5"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B37" s="5"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="5"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B38" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F38" s="9"/>
+      <c r="G38" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+      <c r="L38" s="5"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B39" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F39" s="9"/>
+      <c r="G39" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H39" s="6"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="K39" s="5"/>
+      <c r="L39" s="5"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B40" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H40" s="9"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5"/>
+      <c r="L40" s="5"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B41" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="H41" s="9"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="K41" s="5"/>
+      <c r="L41" s="5"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B42" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F42" s="9"/>
+      <c r="G42" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="K42" s="5"/>
+      <c r="L42" s="5"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B43" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F43" s="9"/>
+      <c r="G43" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="5"/>
+      <c r="L43" s="5"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B44" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="11"/>
+      <c r="H44" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="5"/>
+      <c r="L44" s="5"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B45" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="H45" s="9"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+      <c r="L45" s="5"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B46" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C46" s="12"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5"/>
+      <c r="K46" s="5"/>
+      <c r="L46" s="5"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="B47" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="K47" s="5"/>
+      <c r="L47" s="5"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B48" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K48" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="L48" s="5"/>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B49" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+      <c r="L49" s="5"/>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B50" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="9"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="5"/>
+      <c r="L50" s="5"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B51" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B52" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+      <c r="L52" s="5"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="9"/>
+      <c r="G53" s="9"/>
+      <c r="H53" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="K53" s="5"/>
+      <c r="L53" s="5"/>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B54" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+      <c r="L54" s="5"/>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B55" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="K55" s="5"/>
+      <c r="L55" s="5"/>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="B56" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5"/>
+      <c r="K56" s="5"/>
+      <c r="L56" s="5"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>44</v>
       </c>
+      <c r="B57" s="5"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
+      <c r="F57" s="9"/>
+      <c r="G57" s="9"/>
+      <c r="H57" s="9"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K57" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="L57" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="B58" s="5"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="5"/>
+      <c r="K58" s="5"/>
+      <c r="L58" s="5"/>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="5"/>
+      <c r="K59" s="5"/>
+      <c r="L59" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="G33:G34"/>
+    <mergeCell ref="H38:H39"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>